<commit_message>
tATLAS kNN cleaned_models trained
</commit_message>
<xml_diff>
--- a/datasets/bATLAS_MasterCompiled_reversed.xlsx
+++ b/datasets/bATLAS_MasterCompiled_reversed.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://livejohnshopkins-my.sharepoint.com/personal/lcheng33_jh_edu/Documents/Documents/Academic/1. JHU/1. Research/1. Projects/1. LNPs/Repos/DSPC_Spleen_SORT_FALCON/falcon-lnp-optimization/datasets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="233" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D07B7B5B-D398-4B55-8F55-573C63DEA02D}"/>
+  <xr:revisionPtr revIDLastSave="234" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5BB53DD8-9D63-4C6F-8766-C7FA3ADD2E72}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-3630" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -731,10 +731,10 @@
     </row>
     <row r="2" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="B2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -773,60 +773,60 @@
         <v>790.1</v>
       </c>
       <c r="O2">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="P2">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="Q2">
-        <v>16.66667</v>
+        <v>50</v>
       </c>
       <c r="R2">
         <v>3.75</v>
       </c>
       <c r="S2">
-        <v>24.888887889999999</v>
+        <v>14.518518520000001</v>
       </c>
       <c r="T2">
-        <v>49.999997999999998</v>
+        <v>35</v>
       </c>
       <c r="U2">
-        <v>10.000002</v>
+        <v>35</v>
       </c>
       <c r="V2">
-        <v>38.5</v>
+        <v>28.875</v>
       </c>
       <c r="W2">
-        <v>1.126666682</v>
+        <v>0.96166666700000003</v>
       </c>
       <c r="X2">
-        <v>0.37333331800000003</v>
+        <v>0.163333333</v>
       </c>
       <c r="Y2">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="Z2">
-        <v>3.0000007200000001</v>
+        <v>24</v>
       </c>
       <c r="AA2">
-        <v>11.55000046</v>
+        <v>19.8</v>
       </c>
       <c r="AB2">
-        <v>0.33800001800000001</v>
+        <v>0.65942857099999996</v>
       </c>
       <c r="AC2">
         <v>0.112</v>
       </c>
       <c r="AD2">
-        <v>-1.3846974379999999</v>
+        <v>-1.046034906</v>
       </c>
       <c r="AE2">
-        <v>0.35387085800000001</v>
+        <v>1.039752056</v>
       </c>
     </row>
     <row r="3" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="B3" t="s">
         <v>36</v>
@@ -871,57 +871,57 @@
         <v>5</v>
       </c>
       <c r="P3">
-        <v>40</v>
+        <v>70</v>
       </c>
       <c r="Q3">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="R3">
         <v>3.75</v>
       </c>
       <c r="S3">
-        <v>11.946666670000001</v>
+        <v>23.229629630000002</v>
       </c>
       <c r="T3">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="U3">
-        <v>4</v>
+        <v>35</v>
       </c>
       <c r="V3">
-        <v>57.75</v>
+        <v>28.875</v>
       </c>
       <c r="W3">
-        <v>1.9812000000000001</v>
+        <v>0.86366666700000005</v>
       </c>
       <c r="X3">
-        <v>0.26879999999999998</v>
+        <v>0.261333333</v>
       </c>
       <c r="Y3">
         <v>15</v>
       </c>
       <c r="Z3">
-        <v>1.6666666670000001</v>
+        <v>15</v>
       </c>
       <c r="AA3">
-        <v>24.0625</v>
+        <v>12.375</v>
       </c>
       <c r="AB3">
-        <v>0.82550000000000001</v>
+        <v>0.37014285699999999</v>
       </c>
       <c r="AC3">
         <v>0.112</v>
       </c>
       <c r="AD3">
-        <v>-0.86239050900000003</v>
+        <v>-0.92770153600000005</v>
       </c>
       <c r="AE3">
-        <v>-0.103045105</v>
+        <v>0.80454635299999999</v>
       </c>
     </row>
     <row r="4" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="B4" t="s">
         <v>36</v>
@@ -963,60 +963,60 @@
         <v>790.1</v>
       </c>
       <c r="O4">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="P4">
         <v>55</v>
       </c>
       <c r="Q4">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="R4">
         <v>3.75</v>
       </c>
       <c r="S4">
-        <v>21.902222219999999</v>
+        <v>6.0839506170000002</v>
       </c>
       <c r="T4">
-        <v>49.5</v>
+        <v>22</v>
       </c>
       <c r="U4">
-        <v>5.5</v>
+        <v>33</v>
       </c>
       <c r="V4">
         <v>43.3125</v>
       </c>
       <c r="W4">
-        <v>1.3179000000000001</v>
+        <v>1.584833333</v>
       </c>
       <c r="X4">
-        <v>0.36959999999999998</v>
+        <v>0.102666667</v>
       </c>
       <c r="Y4">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="Z4">
-        <v>1.6666666670000001</v>
+        <v>36</v>
       </c>
       <c r="AA4">
-        <v>13.125</v>
+        <v>47.25</v>
       </c>
       <c r="AB4">
-        <v>0.39936363600000002</v>
+        <v>1.728909091</v>
       </c>
       <c r="AC4">
         <v>0.112</v>
       </c>
       <c r="AD4">
-        <v>-1.0534589240000001</v>
+        <v>-1.602580001</v>
       </c>
       <c r="AE4">
-        <v>-8.3763707000000007E-2</v>
+        <v>0.72410424799999995</v>
       </c>
     </row>
     <row r="5" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="B5" t="s">
         <v>36</v>
@@ -1058,60 +1058,60 @@
         <v>790.1</v>
       </c>
       <c r="O5">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="P5">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="Q5">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="R5">
         <v>3.75</v>
       </c>
       <c r="S5">
-        <v>41.813333329999999</v>
+        <v>7.6049382720000001</v>
       </c>
       <c r="T5">
-        <v>63</v>
+        <v>27.5</v>
       </c>
       <c r="U5">
-        <v>7</v>
+        <v>27.5</v>
       </c>
       <c r="V5">
-        <v>28.875</v>
+        <v>43.3125</v>
       </c>
       <c r="W5">
-        <v>0.65459999999999996</v>
+        <v>1.559166667</v>
       </c>
       <c r="X5">
-        <v>0.47039999999999998</v>
+        <v>0.12833333299999999</v>
       </c>
       <c r="Y5">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="Z5">
-        <v>1.6666666670000001</v>
+        <v>24</v>
       </c>
       <c r="AA5">
-        <v>6.875</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="AB5">
-        <v>0.155857143</v>
+        <v>1.360727273</v>
       </c>
       <c r="AC5">
         <v>0.112</v>
       </c>
       <c r="AD5">
-        <v>-0.47433730600000001</v>
+        <v>-1.6441773669999999</v>
       </c>
       <c r="AE5">
-        <v>-0.373801314</v>
+        <v>0.687393323</v>
       </c>
     </row>
     <row r="6" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="B6" t="s">
         <v>36</v>
@@ -1153,63 +1153,63 @@
         <v>790.1</v>
       </c>
       <c r="O6">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="P6">
-        <v>40</v>
+        <v>70</v>
       </c>
       <c r="Q6">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="R6">
         <v>3.75</v>
       </c>
       <c r="S6">
-        <v>9.2918518520000006</v>
+        <v>11.61481481</v>
       </c>
       <c r="T6">
         <v>28</v>
       </c>
       <c r="U6">
-        <v>12</v>
+        <v>42</v>
       </c>
       <c r="V6">
-        <v>57.75</v>
+        <v>28.875</v>
       </c>
       <c r="W6">
-        <v>2.0409333329999999</v>
+        <v>0.99433333300000004</v>
       </c>
       <c r="X6">
-        <v>0.20906666700000001</v>
+        <v>0.13066666699999999</v>
       </c>
       <c r="Y6">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="Z6">
-        <v>6.4285714289999998</v>
+        <v>36</v>
       </c>
       <c r="AA6">
-        <v>30.9375</v>
+        <v>24.75</v>
       </c>
       <c r="AB6">
-        <v>1.093357143</v>
+        <v>0.85228571399999997</v>
       </c>
       <c r="AC6">
         <v>0.112</v>
       </c>
       <c r="AD6">
-        <v>-1.499651954</v>
+        <v>-1.1834290380000001</v>
       </c>
       <c r="AE6">
-        <v>-5.6782370999999998E-2</v>
+        <v>0.58754348199999995</v>
       </c>
     </row>
     <row r="7" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="B7" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -1251,57 +1251,57 @@
         <v>5</v>
       </c>
       <c r="P7">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="Q7">
-        <v>30</v>
+        <v>16.66667</v>
       </c>
       <c r="R7">
         <v>3.75</v>
       </c>
       <c r="S7">
-        <v>17.035061729999999</v>
+        <v>24.888887889999999</v>
       </c>
       <c r="T7">
+        <v>49.999997999999998</v>
+      </c>
+      <c r="U7">
+        <v>10.000002</v>
+      </c>
+      <c r="V7">
         <v>38.5</v>
       </c>
-      <c r="U7">
-        <v>16.5</v>
-      </c>
-      <c r="V7">
-        <v>43.3125</v>
-      </c>
       <c r="W7">
-        <v>1.4000333330000001</v>
+        <v>1.126666682</v>
       </c>
       <c r="X7">
-        <v>0.28746666700000001</v>
+        <v>0.37333331800000003</v>
       </c>
       <c r="Y7">
         <v>15</v>
       </c>
       <c r="Z7">
-        <v>6.4285714289999998</v>
+        <v>3.0000007200000001</v>
       </c>
       <c r="AA7">
-        <v>16.875</v>
+        <v>11.55000046</v>
       </c>
       <c r="AB7">
-        <v>0.54546753199999998</v>
+        <v>0.33800001800000001</v>
       </c>
       <c r="AC7">
         <v>0.112</v>
       </c>
       <c r="AD7">
-        <v>-1.494572429</v>
+        <v>-1.3846974379999999</v>
       </c>
       <c r="AE7">
-        <v>6.5647288999999998E-2</v>
+        <v>0.35387085800000001</v>
       </c>
     </row>
     <row r="8" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="B8" t="s">
         <v>36</v>
@@ -1343,7 +1343,7 @@
         <v>790.1</v>
       </c>
       <c r="O8">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="P8">
         <v>70</v>
@@ -1355,7 +1355,7 @@
         <v>3.75</v>
       </c>
       <c r="S8">
-        <v>32.521481479999998</v>
+        <v>20.32592593</v>
       </c>
       <c r="T8">
         <v>49</v>
@@ -1367,42 +1367,42 @@
         <v>28.875</v>
       </c>
       <c r="W8">
-        <v>0.75913333299999997</v>
+        <v>0.89633333299999995</v>
       </c>
       <c r="X8">
-        <v>0.36586666699999998</v>
+        <v>0.22866666699999999</v>
       </c>
       <c r="Y8">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="Z8">
-        <v>6.4285714289999998</v>
+        <v>10.28571429</v>
       </c>
       <c r="AA8">
-        <v>8.8392857140000007</v>
+        <v>14.14285714</v>
       </c>
       <c r="AB8">
-        <v>0.232387755</v>
+        <v>0.43902040799999997</v>
       </c>
       <c r="AC8">
         <v>0.112</v>
       </c>
       <c r="AD8">
-        <v>-0.98012685099999997</v>
+        <v>-0.94615079800000002</v>
       </c>
       <c r="AE8">
-        <v>0.18694481600000001</v>
+        <v>0.32683693800000002</v>
       </c>
     </row>
     <row r="9" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>7</v>
+        <v>39</v>
       </c>
       <c r="B9" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="C9">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D9" t="s">
         <v>34</v>
@@ -1438,66 +1438,66 @@
         <v>790.1</v>
       </c>
       <c r="O9">
-        <v>5</v>
+        <v>9.8785700550000008</v>
       </c>
       <c r="P9">
-        <v>40</v>
+        <v>53.934274090000002</v>
       </c>
       <c r="Q9">
-        <v>50</v>
+        <v>45.397458380000003</v>
       </c>
       <c r="R9">
-        <v>3.75</v>
+        <v>2.1242556929999998</v>
       </c>
       <c r="S9">
-        <v>6.6370370369999998</v>
+        <v>11.37354028</v>
       </c>
       <c r="T9">
-        <v>20</v>
+        <v>29.449484460000001</v>
       </c>
       <c r="U9">
-        <v>20</v>
+        <v>24.484789630000002</v>
       </c>
       <c r="V9">
-        <v>57.75</v>
+        <v>45.087172109999997</v>
       </c>
       <c r="W9">
-        <v>2.100666667</v>
+        <v>0.86725759400000002</v>
       </c>
       <c r="X9">
-        <v>0.14933333300000001</v>
+        <v>0.11129621100000001</v>
       </c>
       <c r="Y9">
-        <v>15</v>
+        <v>29.635710159999999</v>
       </c>
       <c r="Z9">
-        <v>15</v>
+        <v>24.639620770000001</v>
       </c>
       <c r="AA9">
-        <v>43.3125</v>
+        <v>45.37228374</v>
       </c>
       <c r="AB9">
-        <v>1.5754999999999999</v>
+        <v>0.87274175300000001</v>
       </c>
       <c r="AC9">
         <v>0.112</v>
       </c>
       <c r="AD9">
-        <v>-1.426921608</v>
+        <v>-0.521548083</v>
       </c>
       <c r="AE9">
-        <v>-3.8710412E-2</v>
+        <v>0.32570661499999998</v>
       </c>
     </row>
     <row r="10" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>8</v>
+        <v>42</v>
       </c>
       <c r="B10" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="C10">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D10" t="s">
         <v>34</v>
@@ -1533,66 +1533,66 @@
         <v>790.1</v>
       </c>
       <c r="O10">
-        <v>5</v>
+        <v>8.0134155969999998</v>
       </c>
       <c r="P10">
-        <v>55</v>
+        <v>61.289618140000002</v>
       </c>
       <c r="Q10">
-        <v>50</v>
+        <v>68.597296510000007</v>
       </c>
       <c r="R10">
-        <v>3.75</v>
+        <v>7.9893410310000004</v>
       </c>
       <c r="S10">
-        <v>12.16790123</v>
+        <v>2.8993099089999999</v>
       </c>
       <c r="T10">
-        <v>27.5</v>
+        <v>19.246597049999998</v>
       </c>
       <c r="U10">
-        <v>27.5</v>
+        <v>42.043021090000003</v>
       </c>
       <c r="V10">
-        <v>43.3125</v>
+        <v>35.617677440000001</v>
       </c>
       <c r="W10">
-        <v>1.482166667</v>
+        <v>3.0030373350000001</v>
       </c>
       <c r="X10">
-        <v>0.20533333300000001</v>
+        <v>8.9667085999999993E-2</v>
       </c>
       <c r="Y10">
-        <v>15</v>
+        <v>24.040246790000001</v>
       </c>
       <c r="Z10">
-        <v>15</v>
+        <v>52.514457489999998</v>
       </c>
       <c r="AA10">
-        <v>23.625</v>
+        <v>44.488786939999997</v>
       </c>
       <c r="AB10">
-        <v>0.80845454500000002</v>
+        <v>3.7509882110000001</v>
       </c>
       <c r="AC10">
         <v>0.112</v>
       </c>
       <c r="AD10">
-        <v>-0.66039868000000002</v>
+        <v>-0.44016229200000001</v>
       </c>
       <c r="AE10">
-        <v>0.21984514999999999</v>
+        <v>0.31605474099999997</v>
       </c>
     </row>
     <row r="11" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>9</v>
+        <v>41</v>
       </c>
       <c r="B11" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="C11">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D11" t="s">
         <v>34</v>
@@ -1628,66 +1628,66 @@
         <v>790.1</v>
       </c>
       <c r="O11">
-        <v>5</v>
+        <v>9.8222594450000003</v>
       </c>
       <c r="P11">
-        <v>70</v>
+        <v>50.262318860000001</v>
       </c>
       <c r="Q11">
-        <v>50</v>
+        <v>68.686957550000002</v>
       </c>
       <c r="R11">
-        <v>3.75</v>
+        <v>8.9776491309999997</v>
       </c>
       <c r="S11">
-        <v>23.229629630000002</v>
+        <v>1.339692087</v>
       </c>
       <c r="T11">
-        <v>35</v>
+        <v>15.738661240000001</v>
       </c>
       <c r="U11">
-        <v>35</v>
+        <v>34.523657620000002</v>
       </c>
       <c r="V11">
-        <v>28.875</v>
+        <v>45.27240664</v>
       </c>
       <c r="W11">
-        <v>0.86366666700000005</v>
+        <v>4.4054535699999997</v>
       </c>
       <c r="X11">
-        <v>0.261333333</v>
+        <v>5.9820929000000002E-2</v>
       </c>
       <c r="Y11">
-        <v>15</v>
+        <v>29.46677833</v>
       </c>
       <c r="Z11">
-        <v>15</v>
+        <v>64.637071140000003</v>
       </c>
       <c r="AA11">
-        <v>12.375</v>
+        <v>84.761464200000006</v>
       </c>
       <c r="AB11">
-        <v>0.37014285699999999</v>
+        <v>8.2481299920000009</v>
       </c>
       <c r="AC11">
         <v>0.112</v>
       </c>
       <c r="AD11">
-        <v>-0.92770153600000005</v>
+        <v>-0.98133603700000005</v>
       </c>
       <c r="AE11">
-        <v>0.80454635299999999</v>
+        <v>0.25767163999999998</v>
       </c>
     </row>
     <row r="12" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="B12" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="C12">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D12" t="s">
         <v>34</v>
@@ -1723,60 +1723,60 @@
         <v>790.1</v>
       </c>
       <c r="O12">
-        <v>5</v>
+        <v>8.0143888000000008</v>
       </c>
       <c r="P12">
-        <v>40</v>
+        <v>70.060370489999997</v>
       </c>
       <c r="Q12">
-        <v>60</v>
+        <v>56.916265009999996</v>
       </c>
       <c r="R12">
-        <v>3.75</v>
+        <v>2.0345911409999999</v>
       </c>
       <c r="S12">
-        <v>5.3096296299999999</v>
+        <v>23.082804060000001</v>
       </c>
       <c r="T12">
-        <v>16</v>
+        <v>30.184624360000001</v>
       </c>
       <c r="U12">
-        <v>24</v>
+        <v>39.875746130000003</v>
       </c>
       <c r="V12">
-        <v>57.75</v>
+        <v>29.33048046</v>
       </c>
       <c r="W12">
-        <v>2.1305333329999998</v>
+        <v>0.46854036799999998</v>
       </c>
       <c r="X12">
-        <v>0.119466667</v>
+        <v>0.14060868200000001</v>
       </c>
       <c r="Y12">
-        <v>15</v>
+        <v>24.0431664</v>
       </c>
       <c r="Z12">
-        <v>22.5</v>
+        <v>31.762502269999999</v>
       </c>
       <c r="AA12">
-        <v>54.140625</v>
+        <v>23.362809290000001</v>
       </c>
       <c r="AB12">
-        <v>1.9973749999999999</v>
+        <v>0.37320968100000002</v>
       </c>
       <c r="AC12">
         <v>0.112</v>
       </c>
       <c r="AD12">
-        <v>-1.13079603</v>
+        <v>-0.28279924400000001</v>
       </c>
       <c r="AE12">
-        <v>-2.9998753999999999E-2</v>
+        <v>0.25156461699999999</v>
       </c>
     </row>
     <row r="13" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B13" t="s">
         <v>36</v>
@@ -1824,60 +1824,60 @@
         <v>55</v>
       </c>
       <c r="Q13">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="R13">
         <v>3.75</v>
       </c>
       <c r="S13">
-        <v>9.7343209880000003</v>
+        <v>12.16790123</v>
       </c>
       <c r="T13">
-        <v>22</v>
+        <v>27.5</v>
       </c>
       <c r="U13">
-        <v>33</v>
+        <v>27.5</v>
       </c>
       <c r="V13">
         <v>43.3125</v>
       </c>
       <c r="W13">
-        <v>1.5232333330000001</v>
+        <v>1.482166667</v>
       </c>
       <c r="X13">
-        <v>0.16426666700000001</v>
+        <v>0.20533333300000001</v>
       </c>
       <c r="Y13">
         <v>15</v>
       </c>
       <c r="Z13">
-        <v>22.5</v>
+        <v>15</v>
       </c>
       <c r="AA13">
-        <v>29.53125</v>
+        <v>23.625</v>
       </c>
       <c r="AB13">
-        <v>1.0385681819999999</v>
+        <v>0.80845454500000002</v>
       </c>
       <c r="AC13">
         <v>0.112</v>
       </c>
       <c r="AD13">
-        <v>-0.98085248899999999</v>
+        <v>-0.66039868000000002</v>
       </c>
       <c r="AE13">
-        <v>6.4326631999999995E-2</v>
+        <v>0.21984514999999999</v>
       </c>
     </row>
     <row r="14" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="B14" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="C14">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D14" t="s">
         <v>34</v>
@@ -1913,60 +1913,60 @@
         <v>790.1</v>
       </c>
       <c r="O14">
-        <v>5</v>
+        <v>8.0118209999999994</v>
       </c>
       <c r="P14">
-        <v>70</v>
+        <v>49.06841884</v>
       </c>
       <c r="Q14">
-        <v>60</v>
+        <v>71.666191310000002</v>
       </c>
       <c r="R14">
-        <v>3.75</v>
+        <v>2.814452143</v>
       </c>
       <c r="S14">
-        <v>18.583703700000001</v>
+        <v>4.5195117920000003</v>
       </c>
       <c r="T14">
-        <v>28</v>
+        <v>13.90295192</v>
       </c>
       <c r="U14">
-        <v>42</v>
+        <v>35.16546692</v>
       </c>
       <c r="V14">
-        <v>28.875</v>
+        <v>49.498136180000003</v>
       </c>
       <c r="W14">
-        <v>0.91593333300000002</v>
+        <v>1.368660263</v>
       </c>
       <c r="X14">
-        <v>0.20906666700000001</v>
+        <v>6.4784715000000007E-2</v>
       </c>
       <c r="Y14">
-        <v>15</v>
+        <v>24.035463</v>
       </c>
       <c r="Z14">
-        <v>22.5</v>
+        <v>60.794159669999999</v>
       </c>
       <c r="AA14">
-        <v>15.46875</v>
+        <v>85.572519229999997</v>
       </c>
       <c r="AB14">
-        <v>0.49067857100000001</v>
+        <v>2.366143772</v>
       </c>
       <c r="AC14">
         <v>0.112</v>
       </c>
       <c r="AD14">
-        <v>-0.92192735599999998</v>
+        <v>-1.0082255200000001</v>
       </c>
       <c r="AE14">
-        <v>3.1071825000000001E-2</v>
+        <v>0.20298074199999999</v>
       </c>
     </row>
     <row r="15" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="B15" t="s">
         <v>36</v>
@@ -2008,66 +2008,66 @@
         <v>790.1</v>
       </c>
       <c r="O15">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="P15">
-        <v>40</v>
+        <v>70</v>
       </c>
       <c r="Q15">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="R15">
         <v>3.75</v>
       </c>
       <c r="S15">
-        <v>7.4666666670000001</v>
+        <v>32.521481479999998</v>
       </c>
       <c r="T15">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="U15">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="V15">
-        <v>57.75</v>
+        <v>28.875</v>
       </c>
       <c r="W15">
-        <v>2.0819999999999999</v>
+        <v>0.75913333299999997</v>
       </c>
       <c r="X15">
-        <v>0.16800000000000001</v>
+        <v>0.36586666699999998</v>
       </c>
       <c r="Y15">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="Z15">
-        <v>2.6666666669999999</v>
+        <v>6.4285714289999998</v>
       </c>
       <c r="AA15">
-        <v>38.5</v>
+        <v>8.8392857140000007</v>
       </c>
       <c r="AB15">
-        <v>1.3879999999999999</v>
+        <v>0.232387755</v>
       </c>
       <c r="AC15">
         <v>0.112</v>
       </c>
       <c r="AD15">
-        <v>-0.97501314800000005</v>
+        <v>-0.98012685099999997</v>
       </c>
       <c r="AE15">
-        <v>-0.10758258699999999</v>
+        <v>0.18694481600000001</v>
       </c>
     </row>
     <row r="16" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="B16" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="C16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D16" t="s">
         <v>34</v>
@@ -2103,60 +2103,60 @@
         <v>790.1</v>
       </c>
       <c r="O16">
-        <v>8</v>
+        <v>4.9193146280000004</v>
       </c>
       <c r="P16">
-        <v>55</v>
+        <v>63.391985609999999</v>
       </c>
       <c r="Q16">
-        <v>10</v>
+        <v>71.982948539999995</v>
       </c>
       <c r="R16">
-        <v>3.75</v>
+        <v>3.8245767829999999</v>
       </c>
       <c r="S16">
-        <v>13.688888889999999</v>
+        <v>9.6269650070000008</v>
       </c>
       <c r="T16">
-        <v>49.5</v>
+        <v>17.760565230000001</v>
       </c>
       <c r="U16">
-        <v>5.5</v>
+        <v>45.631420370000001</v>
       </c>
       <c r="V16">
-        <v>43.3125</v>
+        <v>35.207912780000001</v>
       </c>
       <c r="W16">
-        <v>1.4564999999999999</v>
+        <v>1.2653143259999999</v>
       </c>
       <c r="X16">
-        <v>0.23100000000000001</v>
+        <v>0.134787293</v>
       </c>
       <c r="Y16">
-        <v>24</v>
+        <v>14.757943879999999</v>
       </c>
       <c r="Z16">
-        <v>2.6666666669999999</v>
+        <v>37.916920580000003</v>
       </c>
       <c r="AA16">
-        <v>21</v>
+        <v>29.255623020000002</v>
       </c>
       <c r="AB16">
-        <v>0.70618181800000002</v>
+        <v>1.0513988480000001</v>
       </c>
       <c r="AC16">
         <v>0.112</v>
       </c>
       <c r="AD16">
-        <v>-0.97648036000000005</v>
+        <v>-0.82873811799999997</v>
       </c>
       <c r="AE16">
-        <v>-0.147864672</v>
+        <v>0.18677010199999999</v>
       </c>
     </row>
     <row r="17" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B17" t="s">
         <v>36</v>
@@ -2201,63 +2201,63 @@
         <v>8</v>
       </c>
       <c r="P17">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="Q17">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="R17">
         <v>3.75</v>
       </c>
       <c r="S17">
-        <v>26.133333329999999</v>
+        <v>10.64691358</v>
       </c>
       <c r="T17">
-        <v>63</v>
+        <v>38.5</v>
       </c>
       <c r="U17">
-        <v>7</v>
+        <v>16.5</v>
       </c>
       <c r="V17">
-        <v>28.875</v>
+        <v>43.3125</v>
       </c>
       <c r="W17">
-        <v>0.83099999999999996</v>
+        <v>1.507833333</v>
       </c>
       <c r="X17">
-        <v>0.29399999999999998</v>
+        <v>0.179666667</v>
       </c>
       <c r="Y17">
         <v>24</v>
       </c>
       <c r="Z17">
-        <v>2.6666666669999999</v>
+        <v>10.28571429</v>
       </c>
       <c r="AA17">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="AB17">
-        <v>0.31657142900000002</v>
+        <v>0.93994805199999998</v>
       </c>
       <c r="AC17">
         <v>0.112</v>
       </c>
       <c r="AD17">
-        <v>-0.54703117499999998</v>
+        <v>-1.057731709</v>
       </c>
       <c r="AE17">
-        <v>-0.227944233</v>
+        <v>0.15188178399999999</v>
       </c>
     </row>
     <row r="18" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="B18" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="C18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D18" t="s">
         <v>34</v>
@@ -2293,60 +2293,60 @@
         <v>790.1</v>
       </c>
       <c r="O18">
-        <v>8</v>
+        <v>9.1947111130000003</v>
       </c>
       <c r="P18">
-        <v>40</v>
+        <v>60.034132290000002</v>
       </c>
       <c r="Q18">
-        <v>30</v>
+        <v>64.34235013</v>
       </c>
       <c r="R18">
-        <v>3.75</v>
+        <v>5.9357415390000003</v>
       </c>
       <c r="S18">
-        <v>5.8074074070000004</v>
+        <v>3.6639151270000001</v>
       </c>
       <c r="T18">
-        <v>28</v>
+        <v>21.4067607</v>
       </c>
       <c r="U18">
-        <v>12</v>
+        <v>38.627371599999996</v>
       </c>
       <c r="V18">
-        <v>57.75</v>
+        <v>37.593597099999997</v>
       </c>
       <c r="W18">
-        <v>2.1193333330000002</v>
+        <v>2.2853526290000001</v>
       </c>
       <c r="X18">
-        <v>0.13066666699999999</v>
+        <v>8.6917982000000005E-2</v>
       </c>
       <c r="Y18">
-        <v>24</v>
+        <v>27.584133340000001</v>
       </c>
       <c r="Z18">
-        <v>10.28571429</v>
+        <v>49.774114990000001</v>
       </c>
       <c r="AA18">
-        <v>49.5</v>
+        <v>48.442023040000002</v>
       </c>
       <c r="AB18">
-        <v>1.8165714289999999</v>
+        <v>2.9448393679999998</v>
       </c>
       <c r="AC18">
         <v>0.112</v>
       </c>
       <c r="AD18">
-        <v>-1.579454849</v>
+        <v>-0.636555184</v>
       </c>
       <c r="AE18">
-        <v>7.5741047000000006E-2</v>
+        <v>8.5604358000000005E-2</v>
       </c>
     </row>
     <row r="19" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B19" t="s">
         <v>36</v>
@@ -2391,7 +2391,7 @@
         <v>8</v>
       </c>
       <c r="P19">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="Q19">
         <v>30</v>
@@ -2400,22 +2400,22 @@
         <v>3.75</v>
       </c>
       <c r="S19">
-        <v>10.64691358</v>
+        <v>5.8074074070000004</v>
       </c>
       <c r="T19">
-        <v>38.5</v>
+        <v>28</v>
       </c>
       <c r="U19">
-        <v>16.5</v>
+        <v>12</v>
       </c>
       <c r="V19">
-        <v>43.3125</v>
+        <v>57.75</v>
       </c>
       <c r="W19">
-        <v>1.507833333</v>
+        <v>2.1193333330000002</v>
       </c>
       <c r="X19">
-        <v>0.179666667</v>
+        <v>0.13066666699999999</v>
       </c>
       <c r="Y19">
         <v>24</v>
@@ -2424,24 +2424,24 @@
         <v>10.28571429</v>
       </c>
       <c r="AA19">
-        <v>27</v>
+        <v>49.5</v>
       </c>
       <c r="AB19">
-        <v>0.93994805199999998</v>
+        <v>1.8165714289999999</v>
       </c>
       <c r="AC19">
         <v>0.112</v>
       </c>
       <c r="AD19">
-        <v>-1.057731709</v>
+        <v>-1.579454849</v>
       </c>
       <c r="AE19">
-        <v>0.15188178399999999</v>
+        <v>7.5741047000000006E-2</v>
       </c>
     </row>
     <row r="20" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A20">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="B20" t="s">
         <v>36</v>
@@ -2483,10 +2483,10 @@
         <v>790.1</v>
       </c>
       <c r="O20">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="P20">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="Q20">
         <v>30</v>
@@ -2495,48 +2495,48 @@
         <v>3.75</v>
       </c>
       <c r="S20">
-        <v>20.32592593</v>
+        <v>17.035061729999999</v>
       </c>
       <c r="T20">
-        <v>49</v>
+        <v>38.5</v>
       </c>
       <c r="U20">
-        <v>21</v>
+        <v>16.5</v>
       </c>
       <c r="V20">
-        <v>28.875</v>
+        <v>43.3125</v>
       </c>
       <c r="W20">
-        <v>0.89633333299999995</v>
+        <v>1.4000333330000001</v>
       </c>
       <c r="X20">
-        <v>0.22866666699999999</v>
+        <v>0.28746666700000001</v>
       </c>
       <c r="Y20">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="Z20">
-        <v>10.28571429</v>
+        <v>6.4285714289999998</v>
       </c>
       <c r="AA20">
-        <v>14.14285714</v>
+        <v>16.875</v>
       </c>
       <c r="AB20">
-        <v>0.43902040799999997</v>
+        <v>0.54546753199999998</v>
       </c>
       <c r="AC20">
         <v>0.112</v>
       </c>
       <c r="AD20">
-        <v>-0.94615079800000002</v>
+        <v>-1.494572429</v>
       </c>
       <c r="AE20">
-        <v>0.32683693800000002</v>
+        <v>6.5647288999999998E-2</v>
       </c>
     </row>
     <row r="21" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="B21" t="s">
         <v>36</v>
@@ -2578,66 +2578,66 @@
         <v>790.1</v>
       </c>
       <c r="O21">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="P21">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="Q21">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="R21">
         <v>3.75</v>
       </c>
       <c r="S21">
-        <v>4.1481481479999998</v>
+        <v>9.7343209880000003</v>
       </c>
       <c r="T21">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="U21">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="V21">
-        <v>57.75</v>
+        <v>43.3125</v>
       </c>
       <c r="W21">
-        <v>2.1566666670000001</v>
+        <v>1.5232333330000001</v>
       </c>
       <c r="X21">
-        <v>9.3333333000000004E-2</v>
+        <v>0.16426666700000001</v>
       </c>
       <c r="Y21">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="Z21">
-        <v>24</v>
+        <v>22.5</v>
       </c>
       <c r="AA21">
-        <v>69.3</v>
+        <v>29.53125</v>
       </c>
       <c r="AB21">
-        <v>2.5880000000000001</v>
+        <v>1.0385681819999999</v>
       </c>
       <c r="AC21">
         <v>0.112</v>
       </c>
       <c r="AD21">
-        <v>-1.5728270799999999</v>
+        <v>-0.98085248899999999</v>
       </c>
       <c r="AE21">
-        <v>4.7581602000000001E-2</v>
+        <v>6.4326631999999995E-2</v>
       </c>
     </row>
     <row r="22" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A22">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="B22" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D22" t="s">
         <v>34</v>
@@ -2673,66 +2673,66 @@
         <v>790.1</v>
       </c>
       <c r="O22">
-        <v>8</v>
+        <v>9.7246731000000004</v>
       </c>
       <c r="P22">
-        <v>55</v>
+        <v>39.727072919999998</v>
       </c>
       <c r="Q22">
-        <v>50</v>
+        <v>39.754325479999999</v>
       </c>
       <c r="R22">
-        <v>3.75</v>
+        <v>3.3175453099999999</v>
       </c>
       <c r="S22">
-        <v>7.6049382720000001</v>
+        <v>4.5951008719999997</v>
       </c>
       <c r="T22">
-        <v>27.5</v>
+        <v>23.93384305</v>
       </c>
       <c r="U22">
-        <v>27.5</v>
+        <v>15.793229869999999</v>
       </c>
       <c r="V22">
-        <v>43.3125</v>
+        <v>58.273345419999998</v>
       </c>
       <c r="W22">
-        <v>1.559166667</v>
+        <v>1.907698871</v>
       </c>
       <c r="X22">
-        <v>0.12833333299999999</v>
+        <v>9.1882795000000003E-2</v>
       </c>
       <c r="Y22">
-        <v>24</v>
+        <v>29.174019300000001</v>
       </c>
       <c r="Z22">
-        <v>24</v>
+        <v>19.251066040000001</v>
       </c>
       <c r="AA22">
-        <v>37.799999999999997</v>
+        <v>71.031956730000005</v>
       </c>
       <c r="AB22">
-        <v>1.360727273</v>
+        <v>2.3253784839999998</v>
       </c>
       <c r="AC22">
         <v>0.112</v>
       </c>
       <c r="AD22">
-        <v>-1.6441773669999999</v>
+        <v>-1.729894179</v>
       </c>
       <c r="AE22">
-        <v>0.687393323</v>
+        <v>6.0491143999999997E-2</v>
       </c>
     </row>
     <row r="23" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A23">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="B23" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D23" t="s">
         <v>34</v>
@@ -2768,60 +2768,60 @@
         <v>790.1</v>
       </c>
       <c r="O23">
-        <v>8</v>
+        <v>8.6798676599999993</v>
       </c>
       <c r="P23">
-        <v>70</v>
+        <v>31.885898820000001</v>
       </c>
       <c r="Q23">
-        <v>50</v>
+        <v>48.747130470000002</v>
       </c>
       <c r="R23">
-        <v>3.75</v>
+        <v>4.9097003340000001</v>
       </c>
       <c r="S23">
-        <v>14.518518520000001</v>
+        <v>2.101882807</v>
       </c>
       <c r="T23">
-        <v>35</v>
+        <v>16.342438120000001</v>
       </c>
       <c r="U23">
-        <v>35</v>
+        <v>15.543460700000001</v>
       </c>
       <c r="V23">
-        <v>28.875</v>
+        <v>64.769902930000001</v>
       </c>
       <c r="W23">
-        <v>0.96166666700000003</v>
+        <v>3.273907125</v>
       </c>
       <c r="X23">
-        <v>0.163333333</v>
+        <v>7.0291127999999994E-2</v>
       </c>
       <c r="Y23">
-        <v>24</v>
+        <v>26.039602980000002</v>
       </c>
       <c r="Z23">
-        <v>24</v>
+        <v>24.766533769999999</v>
       </c>
       <c r="AA23">
-        <v>19.8</v>
+        <v>103.20262769999999</v>
       </c>
       <c r="AB23">
-        <v>0.65942857099999996</v>
+        <v>5.2165558839999999</v>
       </c>
       <c r="AC23">
         <v>0.112</v>
       </c>
       <c r="AD23">
-        <v>-1.046034906</v>
+        <v>-1.271982562</v>
       </c>
       <c r="AE23">
-        <v>1.039752056</v>
+        <v>5.8256938000000001E-2</v>
       </c>
     </row>
     <row r="24" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A24">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B24" t="s">
         <v>36</v>
@@ -2869,54 +2869,54 @@
         <v>40</v>
       </c>
       <c r="Q24">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="R24">
         <v>3.75</v>
       </c>
       <c r="S24">
-        <v>3.3185185189999999</v>
+        <v>4.1481481479999998</v>
       </c>
       <c r="T24">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="U24">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="V24">
         <v>57.75</v>
       </c>
       <c r="W24">
-        <v>2.1753333330000002</v>
+        <v>2.1566666670000001</v>
       </c>
       <c r="X24">
-        <v>7.4666667000000006E-2</v>
+        <v>9.3333333000000004E-2</v>
       </c>
       <c r="Y24">
         <v>24</v>
       </c>
       <c r="Z24">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="AA24">
-        <v>86.625</v>
+        <v>69.3</v>
       </c>
       <c r="AB24">
-        <v>3.2629999999999999</v>
+        <v>2.5880000000000001</v>
       </c>
       <c r="AC24">
         <v>0.112</v>
       </c>
       <c r="AD24">
-        <v>-1.296496973</v>
+        <v>-1.5728270799999999</v>
       </c>
       <c r="AE24">
-        <v>2.9603274999999998E-2</v>
+        <v>4.7581602000000001E-2</v>
       </c>
     </row>
     <row r="25" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A25">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="B25" t="s">
         <v>36</v>
@@ -2958,10 +2958,10 @@
         <v>790.1</v>
       </c>
       <c r="O25">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="P25">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="Q25">
         <v>60</v>
@@ -2970,48 +2970,48 @@
         <v>3.75</v>
       </c>
       <c r="S25">
-        <v>6.0839506170000002</v>
+        <v>18.583703700000001</v>
       </c>
       <c r="T25">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="U25">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="V25">
-        <v>43.3125</v>
+        <v>28.875</v>
       </c>
       <c r="W25">
-        <v>1.584833333</v>
+        <v>0.91593333300000002</v>
       </c>
       <c r="X25">
-        <v>0.102666667</v>
+        <v>0.20906666700000001</v>
       </c>
       <c r="Y25">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="Z25">
-        <v>36</v>
+        <v>22.5</v>
       </c>
       <c r="AA25">
-        <v>47.25</v>
+        <v>15.46875</v>
       </c>
       <c r="AB25">
-        <v>1.728909091</v>
+        <v>0.49067857100000001</v>
       </c>
       <c r="AC25">
         <v>0.112</v>
       </c>
       <c r="AD25">
-        <v>-1.602580001</v>
+        <v>-0.92192735599999998</v>
       </c>
       <c r="AE25">
-        <v>0.72410424799999995</v>
+        <v>3.1071825000000001E-2</v>
       </c>
     </row>
     <row r="26" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A26">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B26" t="s">
         <v>36</v>
@@ -3056,7 +3056,7 @@
         <v>8</v>
       </c>
       <c r="P26">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="Q26">
         <v>60</v>
@@ -3065,22 +3065,22 @@
         <v>3.75</v>
       </c>
       <c r="S26">
-        <v>11.61481481</v>
+        <v>3.3185185189999999</v>
       </c>
       <c r="T26">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="U26">
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="V26">
-        <v>28.875</v>
+        <v>57.75</v>
       </c>
       <c r="W26">
-        <v>0.99433333300000004</v>
+        <v>2.1753333330000002</v>
       </c>
       <c r="X26">
-        <v>0.13066666699999999</v>
+        <v>7.4666667000000006E-2</v>
       </c>
       <c r="Y26">
         <v>24</v>
@@ -3089,30 +3089,30 @@
         <v>36</v>
       </c>
       <c r="AA26">
-        <v>24.75</v>
+        <v>86.625</v>
       </c>
       <c r="AB26">
-        <v>0.85228571399999997</v>
+        <v>3.2629999999999999</v>
       </c>
       <c r="AC26">
         <v>0.112</v>
       </c>
       <c r="AD26">
-        <v>-1.1834290380000001</v>
+        <v>-1.296496973</v>
       </c>
       <c r="AE26">
-        <v>0.58754348199999995</v>
+        <v>2.9603274999999998E-2</v>
       </c>
     </row>
     <row r="27" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A27">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="B27" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C27">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D27" t="s">
         <v>34</v>
@@ -3148,60 +3148,60 @@
         <v>790.1</v>
       </c>
       <c r="O27">
-        <v>4.9193146280000004</v>
+        <v>8.3397915440000006</v>
       </c>
       <c r="P27">
-        <v>63.391985609999999</v>
+        <v>88.847310160000006</v>
       </c>
       <c r="Q27">
-        <v>71.982948539999995</v>
+        <v>53.287020740000003</v>
       </c>
       <c r="R27">
-        <v>3.8245767829999999</v>
+        <v>3.5292883000000002</v>
       </c>
       <c r="S27">
-        <v>9.6269650070000008</v>
+        <v>47.201593709999997</v>
       </c>
       <c r="T27">
-        <v>17.760565230000001</v>
+        <v>41.503225569999998</v>
       </c>
       <c r="U27">
-        <v>45.631420370000001</v>
+        <v>47.344084590000001</v>
       </c>
       <c r="V27">
-        <v>35.207912780000001</v>
+        <v>10.75907926</v>
       </c>
       <c r="W27">
-        <v>1.2653143259999999</v>
+        <v>0.207820112</v>
       </c>
       <c r="X27">
-        <v>0.134787293</v>
+        <v>0.18579046599999999</v>
       </c>
       <c r="Y27">
-        <v>14.757943879999999</v>
+        <v>25.019374630000002</v>
       </c>
       <c r="Z27">
-        <v>37.916920580000003</v>
+        <v>28.54041758</v>
       </c>
       <c r="AA27">
-        <v>29.255623020000002</v>
+        <v>6.4858919049999999</v>
       </c>
       <c r="AB27">
-        <v>1.0513988480000001</v>
+        <v>0.12528012399999999</v>
       </c>
       <c r="AC27">
         <v>0.112</v>
       </c>
       <c r="AD27">
-        <v>-0.82873811799999997</v>
+        <v>-3.5081370000000001E-2</v>
       </c>
       <c r="AE27">
-        <v>0.18677010199999999</v>
+        <v>1.6390416000000001E-2</v>
       </c>
     </row>
     <row r="28" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A28">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B28" t="s">
         <v>47</v>
@@ -3243,63 +3243,63 @@
         <v>790.1</v>
       </c>
       <c r="O28">
-        <v>4.9092153420000004</v>
+        <v>9.215869606</v>
       </c>
       <c r="P28">
-        <v>63.40576591</v>
+        <v>55.488986969999999</v>
       </c>
       <c r="Q28">
-        <v>86.141577170000005</v>
+        <v>76.667440780000007</v>
       </c>
       <c r="R28">
-        <v>5.0137559339999997</v>
+        <v>8.9269824880000002</v>
       </c>
       <c r="S28">
-        <v>3.6420960519999999</v>
+        <v>1.319949933</v>
       </c>
       <c r="T28">
-        <v>8.7870391409999993</v>
+        <v>12.94700074</v>
       </c>
       <c r="U28">
-        <v>54.618726770000002</v>
+        <v>42.541986219999998</v>
       </c>
       <c r="V28">
-        <v>34.759488500000003</v>
+        <v>40.537522690000003</v>
       </c>
       <c r="W28">
-        <v>1.767922387</v>
+        <v>3.9210422550000001</v>
       </c>
       <c r="X28">
-        <v>6.6823196000000001E-2</v>
+        <v>5.2448083E-2</v>
       </c>
       <c r="Y28">
-        <v>14.727646030000001</v>
+        <v>27.647608819999999</v>
       </c>
       <c r="Z28">
-        <v>91.544519320000006</v>
+        <v>90.846074450000003</v>
       </c>
       <c r="AA28">
-        <v>58.259151289999998</v>
+        <v>86.565652700000001</v>
       </c>
       <c r="AB28">
-        <v>2.9631522860000001</v>
+        <v>8.3731703260000003</v>
       </c>
       <c r="AC28">
         <v>0.112</v>
       </c>
       <c r="AD28">
-        <v>-0.22791133399999999</v>
+        <v>-4.4158901E-2</v>
       </c>
       <c r="AE28">
-        <v>-8.5357769999999996E-3</v>
+        <v>-6.8394249999999997E-3</v>
       </c>
     </row>
     <row r="29" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A29">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="B29" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="C29">
         <v>1</v>
@@ -3338,60 +3338,60 @@
         <v>790.1</v>
       </c>
       <c r="O29">
-        <v>9.215869606</v>
+        <v>8.3519640299999995</v>
       </c>
       <c r="P29">
-        <v>55.488986969999999</v>
+        <v>28.682729590000001</v>
       </c>
       <c r="Q29">
-        <v>76.667440780000007</v>
+        <v>38.015069680000003</v>
       </c>
       <c r="R29">
-        <v>8.9269824880000002</v>
+        <v>7.2329083799999996</v>
       </c>
       <c r="S29">
-        <v>1.319949933</v>
+        <v>1.5406609389999999</v>
       </c>
       <c r="T29">
-        <v>12.94700074</v>
+        <v>17.77896995</v>
       </c>
       <c r="U29">
-        <v>42.541986219999998</v>
+        <v>10.903759640000001</v>
       </c>
       <c r="V29">
-        <v>40.537522690000003</v>
+        <v>66.15895759</v>
       </c>
       <c r="W29">
-        <v>3.9210422550000001</v>
+        <v>5.0788407170000003</v>
       </c>
       <c r="X29">
-        <v>5.2448083E-2</v>
+        <v>7.9472110999999998E-2</v>
       </c>
       <c r="Y29">
-        <v>27.647608819999999</v>
+        <v>25.05589209</v>
       </c>
       <c r="Z29">
-        <v>90.846074450000003</v>
+        <v>15.36666217</v>
       </c>
       <c r="AA29">
-        <v>86.565652700000001</v>
+        <v>93.237780749999999</v>
       </c>
       <c r="AB29">
-        <v>8.3731703260000003</v>
+        <v>7.1576072919999998</v>
       </c>
       <c r="AC29">
         <v>0.112</v>
       </c>
       <c r="AD29">
-        <v>-4.4158901E-2</v>
+        <v>-0.63623467199999995</v>
       </c>
       <c r="AE29">
-        <v>-6.8394249999999997E-3</v>
+        <v>-7.9426949999999996E-3</v>
       </c>
     </row>
     <row r="30" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A30">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B30" t="s">
         <v>47</v>
@@ -3433,63 +3433,63 @@
         <v>790.1</v>
       </c>
       <c r="O30">
-        <v>9.1947111130000003</v>
+        <v>4.9092153420000004</v>
       </c>
       <c r="P30">
-        <v>60.034132290000002</v>
+        <v>63.40576591</v>
       </c>
       <c r="Q30">
-        <v>64.34235013</v>
+        <v>86.141577170000005</v>
       </c>
       <c r="R30">
-        <v>5.9357415390000003</v>
+        <v>5.0137559339999997</v>
       </c>
       <c r="S30">
-        <v>3.6639151270000001</v>
+        <v>3.6420960519999999</v>
       </c>
       <c r="T30">
-        <v>21.4067607</v>
+        <v>8.7870391409999993</v>
       </c>
       <c r="U30">
-        <v>38.627371599999996</v>
+        <v>54.618726770000002</v>
       </c>
       <c r="V30">
-        <v>37.593597099999997</v>
+        <v>34.759488500000003</v>
       </c>
       <c r="W30">
-        <v>2.2853526290000001</v>
+        <v>1.767922387</v>
       </c>
       <c r="X30">
-        <v>8.6917982000000005E-2</v>
+        <v>6.6823196000000001E-2</v>
       </c>
       <c r="Y30">
-        <v>27.584133340000001</v>
+        <v>14.727646030000001</v>
       </c>
       <c r="Z30">
-        <v>49.774114990000001</v>
+        <v>91.544519320000006</v>
       </c>
       <c r="AA30">
-        <v>48.442023040000002</v>
+        <v>58.259151289999998</v>
       </c>
       <c r="AB30">
-        <v>2.9448393679999998</v>
+        <v>2.9631522860000001</v>
       </c>
       <c r="AC30">
         <v>0.112</v>
       </c>
       <c r="AD30">
-        <v>-0.636555184</v>
+        <v>-0.22791133399999999</v>
       </c>
       <c r="AE30">
-        <v>8.5604358000000005E-2</v>
+        <v>-8.5357769999999996E-3</v>
       </c>
     </row>
     <row r="31" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A31">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B31" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="C31">
         <v>1</v>
@@ -3528,66 +3528,66 @@
         <v>790.1</v>
       </c>
       <c r="O31">
-        <v>7.6942788709999999</v>
+        <v>8.0831456690000003</v>
       </c>
       <c r="P31">
-        <v>61.632936049999998</v>
+        <v>46.063229249999999</v>
       </c>
       <c r="Q31">
-        <v>78.316335219999999</v>
+        <v>35.192255320000001</v>
       </c>
       <c r="R31">
-        <v>6.6286994740000003</v>
+        <v>8.3008092809999994</v>
       </c>
       <c r="S31">
-        <v>2.5496906479999999</v>
+        <v>3.0795855599999999</v>
       </c>
       <c r="T31">
-        <v>13.364279249999999</v>
+        <v>29.852540000000001</v>
       </c>
       <c r="U31">
-        <v>48.268656810000003</v>
+        <v>16.210689250000001</v>
       </c>
       <c r="V31">
-        <v>35.823826580000002</v>
+        <v>49.459582279999999</v>
       </c>
       <c r="W31">
-        <v>2.4783926809999999</v>
+        <v>4.3393096230000001</v>
       </c>
       <c r="X31">
-        <v>6.4844684999999999E-2</v>
+        <v>0.13787885</v>
       </c>
       <c r="Y31">
-        <v>23.082836610000001</v>
+        <v>24.249437010000001</v>
       </c>
       <c r="Z31">
-        <v>83.369817269999999</v>
+        <v>13.16806167</v>
       </c>
       <c r="AA31">
-        <v>61.875056690000001</v>
+        <v>40.176381139999997</v>
       </c>
       <c r="AB31">
-        <v>4.2806897599999996</v>
+        <v>3.5248530059999998</v>
       </c>
       <c r="AC31">
         <v>0.112</v>
       </c>
       <c r="AD31">
-        <v>-0.49055528799999998</v>
+        <v>-1.1070581829999999</v>
       </c>
       <c r="AE31">
-        <v>-5.7851792999999999E-2</v>
+        <v>-2.8333599000000001E-2</v>
       </c>
     </row>
     <row r="32" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A32">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="B32" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C32">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D32" t="s">
         <v>34</v>
@@ -3623,60 +3623,60 @@
         <v>790.1</v>
       </c>
       <c r="O32">
-        <v>8.6798676599999993</v>
+        <v>5</v>
       </c>
       <c r="P32">
-        <v>31.885898820000001</v>
+        <v>40</v>
       </c>
       <c r="Q32">
-        <v>48.747130470000002</v>
+        <v>60</v>
       </c>
       <c r="R32">
-        <v>4.9097003340000001</v>
+        <v>3.75</v>
       </c>
       <c r="S32">
-        <v>2.101882807</v>
+        <v>5.3096296299999999</v>
       </c>
       <c r="T32">
-        <v>16.342438120000001</v>
+        <v>16</v>
       </c>
       <c r="U32">
-        <v>15.543460700000001</v>
+        <v>24</v>
       </c>
       <c r="V32">
-        <v>64.769902930000001</v>
+        <v>57.75</v>
       </c>
       <c r="W32">
-        <v>3.273907125</v>
+        <v>2.1305333329999998</v>
       </c>
       <c r="X32">
-        <v>7.0291127999999994E-2</v>
+        <v>0.119466667</v>
       </c>
       <c r="Y32">
-        <v>26.039602980000002</v>
+        <v>15</v>
       </c>
       <c r="Z32">
-        <v>24.766533769999999</v>
+        <v>22.5</v>
       </c>
       <c r="AA32">
-        <v>103.20262769999999</v>
+        <v>54.140625</v>
       </c>
       <c r="AB32">
-        <v>5.2165558839999999</v>
+        <v>1.9973749999999999</v>
       </c>
       <c r="AC32">
         <v>0.112</v>
       </c>
       <c r="AD32">
-        <v>-1.271982562</v>
+        <v>-1.13079603</v>
       </c>
       <c r="AE32">
-        <v>5.8256938000000001E-2</v>
+        <v>-2.9998753999999999E-2</v>
       </c>
     </row>
     <row r="33" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A33">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B33" t="s">
         <v>37</v>
@@ -3718,66 +3718,66 @@
         <v>790.1</v>
       </c>
       <c r="O33">
-        <v>9.7246731000000004</v>
+        <v>9.7036068879999995</v>
       </c>
       <c r="P33">
-        <v>39.727072919999998</v>
+        <v>22.115852950000001</v>
       </c>
       <c r="Q33">
-        <v>39.754325479999999</v>
+        <v>49.07019871</v>
       </c>
       <c r="R33">
-        <v>3.3175453099999999</v>
+        <v>8.5277041639999993</v>
       </c>
       <c r="S33">
-        <v>4.5951008719999997</v>
+        <v>0.65246625499999999</v>
       </c>
       <c r="T33">
-        <v>23.93384305</v>
+        <v>11.26355996</v>
       </c>
       <c r="U33">
-        <v>15.793229869999999</v>
+        <v>10.85229299</v>
       </c>
       <c r="V33">
-        <v>58.273345419999998</v>
+        <v>71.242417399999994</v>
       </c>
       <c r="W33">
-        <v>1.907698871</v>
+        <v>6.5983946070000004</v>
       </c>
       <c r="X33">
-        <v>9.1882795000000003E-2</v>
+        <v>4.3335045000000003E-2</v>
       </c>
       <c r="Y33">
-        <v>29.174019300000001</v>
+        <v>29.110820669999999</v>
       </c>
       <c r="Z33">
-        <v>19.251066040000001</v>
+        <v>28.047895700000002</v>
       </c>
       <c r="AA33">
-        <v>71.031956730000005</v>
+        <v>184.1269762</v>
       </c>
       <c r="AB33">
-        <v>2.3253784839999998</v>
+        <v>17.0536387</v>
       </c>
       <c r="AC33">
         <v>0.112</v>
       </c>
       <c r="AD33">
-        <v>-1.729894179</v>
+        <v>-0.33568535599999999</v>
       </c>
       <c r="AE33">
-        <v>6.0491143999999997E-2</v>
+        <v>-3.5648119999999998E-2</v>
       </c>
     </row>
     <row r="34" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A34">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="B34" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C34">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D34" t="s">
         <v>34</v>
@@ -3813,66 +3813,66 @@
         <v>790.1</v>
       </c>
       <c r="O34">
-        <v>8.0831456690000003</v>
+        <v>5</v>
       </c>
       <c r="P34">
-        <v>46.063229249999999</v>
+        <v>40</v>
       </c>
       <c r="Q34">
-        <v>35.192255320000001</v>
+        <v>50</v>
       </c>
       <c r="R34">
-        <v>8.3008092809999994</v>
+        <v>3.75</v>
       </c>
       <c r="S34">
-        <v>3.0795855599999999</v>
+        <v>6.6370370369999998</v>
       </c>
       <c r="T34">
-        <v>29.852540000000001</v>
+        <v>20</v>
       </c>
       <c r="U34">
-        <v>16.210689250000001</v>
+        <v>20</v>
       </c>
       <c r="V34">
-        <v>49.459582279999999</v>
+        <v>57.75</v>
       </c>
       <c r="W34">
-        <v>4.3393096230000001</v>
+        <v>2.100666667</v>
       </c>
       <c r="X34">
-        <v>0.13787885</v>
+        <v>0.14933333300000001</v>
       </c>
       <c r="Y34">
-        <v>24.249437010000001</v>
+        <v>15</v>
       </c>
       <c r="Z34">
-        <v>13.16806167</v>
+        <v>15</v>
       </c>
       <c r="AA34">
-        <v>40.176381139999997</v>
+        <v>43.3125</v>
       </c>
       <c r="AB34">
-        <v>3.5248530059999998</v>
+        <v>1.5754999999999999</v>
       </c>
       <c r="AC34">
         <v>0.112</v>
       </c>
       <c r="AD34">
-        <v>-1.1070581829999999</v>
+        <v>-1.426921608</v>
       </c>
       <c r="AE34">
-        <v>-2.8333599000000001E-2</v>
+        <v>-3.8710412E-2</v>
       </c>
     </row>
     <row r="35" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A35">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="B35" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C35">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D35" t="s">
         <v>34</v>
@@ -3908,63 +3908,63 @@
         <v>790.1</v>
       </c>
       <c r="O35">
-        <v>8.3519640299999995</v>
+        <v>5</v>
       </c>
       <c r="P35">
-        <v>28.682729590000001</v>
+        <v>40</v>
       </c>
       <c r="Q35">
-        <v>38.015069680000003</v>
+        <v>30</v>
       </c>
       <c r="R35">
-        <v>7.2329083799999996</v>
+        <v>3.75</v>
       </c>
       <c r="S35">
-        <v>1.5406609389999999</v>
+        <v>9.2918518520000006</v>
       </c>
       <c r="T35">
-        <v>17.77896995</v>
+        <v>28</v>
       </c>
       <c r="U35">
-        <v>10.903759640000001</v>
+        <v>12</v>
       </c>
       <c r="V35">
-        <v>66.15895759</v>
+        <v>57.75</v>
       </c>
       <c r="W35">
-        <v>5.0788407170000003</v>
+        <v>2.0409333329999999</v>
       </c>
       <c r="X35">
-        <v>7.9472110999999998E-2</v>
+        <v>0.20906666700000001</v>
       </c>
       <c r="Y35">
-        <v>25.05589209</v>
+        <v>15</v>
       </c>
       <c r="Z35">
-        <v>15.36666217</v>
+        <v>6.4285714289999998</v>
       </c>
       <c r="AA35">
-        <v>93.237780749999999</v>
+        <v>30.9375</v>
       </c>
       <c r="AB35">
-        <v>7.1576072919999998</v>
+        <v>1.093357143</v>
       </c>
       <c r="AC35">
         <v>0.112</v>
       </c>
       <c r="AD35">
-        <v>-0.63623467199999995</v>
+        <v>-1.499651954</v>
       </c>
       <c r="AE35">
-        <v>-7.9426949999999996E-3</v>
+        <v>-5.6782370999999998E-2</v>
       </c>
     </row>
     <row r="36" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A36">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="B36" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="C36">
         <v>1</v>
@@ -4003,66 +4003,66 @@
         <v>790.1</v>
       </c>
       <c r="O36">
-        <v>9.7036068879999995</v>
+        <v>7.6942788709999999</v>
       </c>
       <c r="P36">
-        <v>22.115852950000001</v>
+        <v>61.632936049999998</v>
       </c>
       <c r="Q36">
-        <v>49.07019871</v>
+        <v>78.316335219999999</v>
       </c>
       <c r="R36">
-        <v>8.5277041639999993</v>
+        <v>6.6286994740000003</v>
       </c>
       <c r="S36">
-        <v>0.65246625499999999</v>
+        <v>2.5496906479999999</v>
       </c>
       <c r="T36">
-        <v>11.26355996</v>
+        <v>13.364279249999999</v>
       </c>
       <c r="U36">
-        <v>10.85229299</v>
+        <v>48.268656810000003</v>
       </c>
       <c r="V36">
-        <v>71.242417399999994</v>
+        <v>35.823826580000002</v>
       </c>
       <c r="W36">
-        <v>6.5983946070000004</v>
+        <v>2.4783926809999999</v>
       </c>
       <c r="X36">
-        <v>4.3335045000000003E-2</v>
+        <v>6.4844684999999999E-2</v>
       </c>
       <c r="Y36">
-        <v>29.110820669999999</v>
+        <v>23.082836610000001</v>
       </c>
       <c r="Z36">
-        <v>28.047895700000002</v>
+        <v>83.369817269999999</v>
       </c>
       <c r="AA36">
-        <v>184.1269762</v>
+        <v>61.875056690000001</v>
       </c>
       <c r="AB36">
-        <v>17.0536387</v>
+        <v>4.2806897599999996</v>
       </c>
       <c r="AC36">
         <v>0.112</v>
       </c>
       <c r="AD36">
-        <v>-0.33568535599999999</v>
+        <v>-0.49055528799999998</v>
       </c>
       <c r="AE36">
-        <v>-3.5648119999999998E-2</v>
+        <v>-5.7851792999999999E-2</v>
       </c>
     </row>
     <row r="37" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A37">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="B37" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="C37">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D37" t="s">
         <v>34</v>
@@ -4098,66 +4098,66 @@
         <v>790.1</v>
       </c>
       <c r="O37">
-        <v>8.2789758590000009</v>
+        <v>5</v>
       </c>
       <c r="P37">
-        <v>47.573096079999999</v>
+        <v>55</v>
       </c>
       <c r="Q37">
-        <v>35.970323409999999</v>
+        <v>10</v>
       </c>
       <c r="R37">
-        <v>2.8522899449999999</v>
+        <v>3.75</v>
       </c>
       <c r="S37">
-        <v>9.1857578849999992</v>
+        <v>21.902222219999999</v>
       </c>
       <c r="T37">
-        <v>30.460899560000001</v>
+        <v>49.5</v>
       </c>
       <c r="U37">
-        <v>17.112196520000001</v>
+        <v>5.5</v>
       </c>
       <c r="V37">
-        <v>50.931536610000002</v>
+        <v>43.3125</v>
       </c>
       <c r="W37">
-        <v>1.3580064890000001</v>
+        <v>1.3179000000000001</v>
       </c>
       <c r="X37">
-        <v>0.13736082099999999</v>
+        <v>0.36959999999999998</v>
       </c>
       <c r="Y37">
-        <v>24.836927580000001</v>
+        <v>15</v>
       </c>
       <c r="Z37">
-        <v>13.9527851</v>
+        <v>1.6666666670000001</v>
       </c>
       <c r="AA37">
-        <v>41.528086969999997</v>
+        <v>13.125</v>
       </c>
       <c r="AB37">
-        <v>1.107278816</v>
+        <v>0.39936363600000002</v>
       </c>
       <c r="AC37">
         <v>0.112</v>
       </c>
       <c r="AD37">
-        <v>-1.402072242</v>
+        <v>-1.0534589240000001</v>
       </c>
       <c r="AE37">
-        <v>-0.265925034</v>
+        <v>-8.3763707000000007E-2</v>
       </c>
     </row>
     <row r="38" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A38">
-        <v>36</v>
+        <v>1</v>
       </c>
       <c r="B38" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="C38">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D38" t="s">
         <v>34</v>
@@ -4193,66 +4193,66 @@
         <v>790.1</v>
       </c>
       <c r="O38">
-        <v>8.3397915440000006</v>
+        <v>5</v>
       </c>
       <c r="P38">
-        <v>88.847310160000006</v>
+        <v>40</v>
       </c>
       <c r="Q38">
-        <v>53.287020740000003</v>
+        <v>10</v>
       </c>
       <c r="R38">
-        <v>3.5292883000000002</v>
+        <v>3.75</v>
       </c>
       <c r="S38">
-        <v>47.201593709999997</v>
+        <v>11.946666670000001</v>
       </c>
       <c r="T38">
-        <v>41.503225569999998</v>
+        <v>36</v>
       </c>
       <c r="U38">
-        <v>47.344084590000001</v>
+        <v>4</v>
       </c>
       <c r="V38">
-        <v>10.75907926</v>
+        <v>57.75</v>
       </c>
       <c r="W38">
-        <v>0.207820112</v>
+        <v>1.9812000000000001</v>
       </c>
       <c r="X38">
-        <v>0.18579046599999999</v>
+        <v>0.26879999999999998</v>
       </c>
       <c r="Y38">
-        <v>25.019374630000002</v>
+        <v>15</v>
       </c>
       <c r="Z38">
-        <v>28.54041758</v>
+        <v>1.6666666670000001</v>
       </c>
       <c r="AA38">
-        <v>6.4858919049999999</v>
+        <v>24.0625</v>
       </c>
       <c r="AB38">
-        <v>0.12528012399999999</v>
+        <v>0.82550000000000001</v>
       </c>
       <c r="AC38">
         <v>0.112</v>
       </c>
       <c r="AD38">
-        <v>-3.5081370000000001E-2</v>
+        <v>-0.86239050900000003</v>
       </c>
       <c r="AE38">
-        <v>1.6390416000000001E-2</v>
+        <v>-0.103045105</v>
       </c>
     </row>
     <row r="39" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A39">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="B39" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="C39">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D39" t="s">
         <v>34</v>
@@ -4288,66 +4288,66 @@
         <v>790.1</v>
       </c>
       <c r="O39">
-        <v>8.0143888000000008</v>
+        <v>8</v>
       </c>
       <c r="P39">
-        <v>70.060370489999997</v>
+        <v>40</v>
       </c>
       <c r="Q39">
-        <v>56.916265009999996</v>
+        <v>10</v>
       </c>
       <c r="R39">
-        <v>2.0345911409999999</v>
+        <v>3.75</v>
       </c>
       <c r="S39">
-        <v>23.082804060000001</v>
+        <v>7.4666666670000001</v>
       </c>
       <c r="T39">
-        <v>30.184624360000001</v>
+        <v>36</v>
       </c>
       <c r="U39">
-        <v>39.875746130000003</v>
+        <v>4</v>
       </c>
       <c r="V39">
-        <v>29.33048046</v>
+        <v>57.75</v>
       </c>
       <c r="W39">
-        <v>0.46854036799999998</v>
+        <v>2.0819999999999999</v>
       </c>
       <c r="X39">
-        <v>0.14060868200000001</v>
+        <v>0.16800000000000001</v>
       </c>
       <c r="Y39">
-        <v>24.0431664</v>
+        <v>24</v>
       </c>
       <c r="Z39">
-        <v>31.762502269999999</v>
+        <v>2.6666666669999999</v>
       </c>
       <c r="AA39">
-        <v>23.362809290000001</v>
+        <v>38.5</v>
       </c>
       <c r="AB39">
-        <v>0.37320968100000002</v>
+        <v>1.3879999999999999</v>
       </c>
       <c r="AC39">
         <v>0.112</v>
       </c>
       <c r="AD39">
-        <v>-0.28279924400000001</v>
+        <v>-0.97501314800000005</v>
       </c>
       <c r="AE39">
-        <v>0.25156461699999999</v>
+        <v>-0.10758258699999999</v>
       </c>
     </row>
     <row r="40" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A40">
-        <v>38</v>
+        <v>14</v>
       </c>
       <c r="B40" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="C40">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D40" t="s">
         <v>34</v>
@@ -4383,63 +4383,63 @@
         <v>790.1</v>
       </c>
       <c r="O40">
-        <v>8.0118209999999994</v>
+        <v>8</v>
       </c>
       <c r="P40">
-        <v>49.06841884</v>
+        <v>55</v>
       </c>
       <c r="Q40">
-        <v>71.666191310000002</v>
+        <v>10</v>
       </c>
       <c r="R40">
-        <v>2.814452143</v>
+        <v>3.75</v>
       </c>
       <c r="S40">
-        <v>4.5195117920000003</v>
+        <v>13.688888889999999</v>
       </c>
       <c r="T40">
-        <v>13.90295192</v>
+        <v>49.5</v>
       </c>
       <c r="U40">
-        <v>35.16546692</v>
+        <v>5.5</v>
       </c>
       <c r="V40">
-        <v>49.498136180000003</v>
+        <v>43.3125</v>
       </c>
       <c r="W40">
-        <v>1.368660263</v>
+        <v>1.4564999999999999</v>
       </c>
       <c r="X40">
-        <v>6.4784715000000007E-2</v>
+        <v>0.23100000000000001</v>
       </c>
       <c r="Y40">
-        <v>24.035463</v>
+        <v>24</v>
       </c>
       <c r="Z40">
-        <v>60.794159669999999</v>
+        <v>2.6666666669999999</v>
       </c>
       <c r="AA40">
-        <v>85.572519229999997</v>
+        <v>21</v>
       </c>
       <c r="AB40">
-        <v>2.366143772</v>
+        <v>0.70618181800000002</v>
       </c>
       <c r="AC40">
         <v>0.112</v>
       </c>
       <c r="AD40">
-        <v>-1.0082255200000001</v>
+        <v>-0.97648036000000005</v>
       </c>
       <c r="AE40">
-        <v>0.20298074199999999</v>
+        <v>-0.147864672</v>
       </c>
     </row>
     <row r="41" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A41">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B41" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C41">
         <v>2</v>
@@ -4478,66 +4478,66 @@
         <v>790.1</v>
       </c>
       <c r="O41">
-        <v>9.8785700550000008</v>
+        <v>6.7062622530000002</v>
       </c>
       <c r="P41">
-        <v>53.934274090000002</v>
+        <v>58.59190426</v>
       </c>
       <c r="Q41">
-        <v>45.397458380000003</v>
+        <v>24.337806520000001</v>
       </c>
       <c r="R41">
-        <v>2.1242556929999998</v>
+        <v>6.2871595100000004</v>
       </c>
       <c r="S41">
-        <v>11.37354028</v>
+        <v>9.4796660460000002</v>
       </c>
       <c r="T41">
-        <v>29.449484460000001</v>
+        <v>44.331919970000001</v>
       </c>
       <c r="U41">
-        <v>24.484789630000002</v>
+        <v>14.25998429</v>
       </c>
       <c r="V41">
-        <v>45.087172109999997</v>
+        <v>38.804702710000001</v>
       </c>
       <c r="W41">
-        <v>0.86725759400000002</v>
+        <v>2.3566000640000002</v>
       </c>
       <c r="X41">
-        <v>0.11129621100000001</v>
+        <v>0.246792965</v>
       </c>
       <c r="Y41">
-        <v>29.635710159999999</v>
+        <v>20.118786759999999</v>
       </c>
       <c r="Z41">
-        <v>24.639620770000001</v>
+        <v>6.4714901449999997</v>
       </c>
       <c r="AA41">
-        <v>45.37228374</v>
+        <v>17.61041569</v>
       </c>
       <c r="AB41">
-        <v>0.87274175300000001</v>
+        <v>1.069476219</v>
       </c>
       <c r="AC41">
         <v>0.112</v>
       </c>
       <c r="AD41">
-        <v>-0.521548083</v>
+        <v>-0.629023471</v>
       </c>
       <c r="AE41">
-        <v>0.32570661499999998</v>
+        <v>-0.15897987199999999</v>
       </c>
     </row>
     <row r="42" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A42">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="B42" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="C42">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D42" t="s">
         <v>34</v>
@@ -4573,60 +4573,60 @@
         <v>790.1</v>
       </c>
       <c r="O42">
-        <v>4.9056310139999999</v>
+        <v>8</v>
       </c>
       <c r="P42">
-        <v>36.437753440000002</v>
+        <v>70</v>
       </c>
       <c r="Q42">
-        <v>33.968589559999998</v>
+        <v>10</v>
       </c>
       <c r="R42">
-        <v>6.5750179839999996</v>
+        <v>3.75</v>
       </c>
       <c r="S42">
-        <v>4.3813492370000002</v>
+        <v>26.133333329999999</v>
       </c>
       <c r="T42">
-        <v>24.060362529999999</v>
+        <v>63</v>
       </c>
       <c r="U42">
-        <v>12.377390910000001</v>
+        <v>7</v>
       </c>
       <c r="V42">
-        <v>59.383017420000002</v>
+        <v>28.875</v>
       </c>
       <c r="W42">
-        <v>3.996122518</v>
+        <v>0.83099999999999996</v>
       </c>
       <c r="X42">
-        <v>0.183106624</v>
+        <v>0.29399999999999998</v>
       </c>
       <c r="Y42">
-        <v>14.71689304</v>
+        <v>24</v>
       </c>
       <c r="Z42">
-        <v>7.5708226749999996</v>
+        <v>2.6666666669999999</v>
       </c>
       <c r="AA42">
-        <v>36.322541479999998</v>
+        <v>11</v>
       </c>
       <c r="AB42">
-        <v>2.4442901730000002</v>
+        <v>0.31657142900000002</v>
       </c>
       <c r="AC42">
         <v>0.112</v>
       </c>
       <c r="AD42">
-        <v>-1.613734727</v>
+        <v>-0.54703117499999998</v>
       </c>
       <c r="AE42">
-        <v>-0.27725127399999999</v>
+        <v>-0.227944233</v>
       </c>
     </row>
     <row r="43" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A43">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B43" t="s">
         <v>47</v>
@@ -4668,63 +4668,63 @@
         <v>790.1</v>
       </c>
       <c r="O43">
-        <v>9.8222594450000003</v>
+        <v>6.2861622239999999</v>
       </c>
       <c r="P43">
-        <v>50.262318860000001</v>
+        <v>30.096331939999999</v>
       </c>
       <c r="Q43">
-        <v>68.686957550000002</v>
+        <v>47.51337024</v>
       </c>
       <c r="R43">
-        <v>8.9776491309999997</v>
+        <v>8.5863137839999997</v>
       </c>
       <c r="S43">
-        <v>1.339692087</v>
+        <v>1.5630278559999999</v>
       </c>
       <c r="T43">
-        <v>15.738661240000001</v>
+        <v>15.79655032</v>
       </c>
       <c r="U43">
-        <v>34.523657620000002</v>
+        <v>14.299781619999999</v>
       </c>
       <c r="V43">
-        <v>45.27240664</v>
+        <v>63.90151977</v>
       </c>
       <c r="W43">
-        <v>4.4054535699999997</v>
+        <v>5.9083330370000002</v>
       </c>
       <c r="X43">
-        <v>5.9820929000000002E-2</v>
+        <v>9.3815250000000003E-2</v>
       </c>
       <c r="Y43">
-        <v>29.46677833</v>
+        <v>18.858486670000001</v>
       </c>
       <c r="Z43">
-        <v>64.637071140000003</v>
+        <v>17.07159068</v>
       </c>
       <c r="AA43">
-        <v>84.761464200000006</v>
+        <v>76.287919500000001</v>
       </c>
       <c r="AB43">
-        <v>8.2481299920000009</v>
+        <v>7.053579268</v>
       </c>
       <c r="AC43">
         <v>0.112</v>
       </c>
       <c r="AD43">
-        <v>-0.98133603700000005</v>
+        <v>-1.5549625840000001</v>
       </c>
       <c r="AE43">
-        <v>0.25767163999999998</v>
+        <v>-0.24728119900000001</v>
       </c>
     </row>
     <row r="44" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A44">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="B44" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C44">
         <v>2</v>
@@ -4763,60 +4763,60 @@
         <v>790.1</v>
       </c>
       <c r="O44">
-        <v>8.0134155969999998</v>
+        <v>8.2789758590000009</v>
       </c>
       <c r="P44">
-        <v>61.289618140000002</v>
+        <v>47.573096079999999</v>
       </c>
       <c r="Q44">
-        <v>68.597296510000007</v>
+        <v>35.970323409999999</v>
       </c>
       <c r="R44">
-        <v>7.9893410310000004</v>
+        <v>2.8522899449999999</v>
       </c>
       <c r="S44">
-        <v>2.8993099089999999</v>
+        <v>9.1857578849999992</v>
       </c>
       <c r="T44">
-        <v>19.246597049999998</v>
+        <v>30.460899560000001</v>
       </c>
       <c r="U44">
-        <v>42.043021090000003</v>
+        <v>17.112196520000001</v>
       </c>
       <c r="V44">
-        <v>35.617677440000001</v>
+        <v>50.931536610000002</v>
       </c>
       <c r="W44">
-        <v>3.0030373350000001</v>
+        <v>1.3580064890000001</v>
       </c>
       <c r="X44">
-        <v>8.9667085999999993E-2</v>
+        <v>0.13736082099999999</v>
       </c>
       <c r="Y44">
-        <v>24.040246790000001</v>
+        <v>24.836927580000001</v>
       </c>
       <c r="Z44">
-        <v>52.514457489999998</v>
+        <v>13.9527851</v>
       </c>
       <c r="AA44">
-        <v>44.488786939999997</v>
+        <v>41.528086969999997</v>
       </c>
       <c r="AB44">
-        <v>3.7509882110000001</v>
+        <v>1.107278816</v>
       </c>
       <c r="AC44">
         <v>0.112</v>
       </c>
       <c r="AD44">
-        <v>-0.44016229200000001</v>
+        <v>-1.402072242</v>
       </c>
       <c r="AE44">
-        <v>0.31605474099999997</v>
+        <v>-0.265925034</v>
       </c>
     </row>
     <row r="45" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A45">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B45" t="s">
         <v>47</v>
@@ -4858,66 +4858,66 @@
         <v>790.1</v>
       </c>
       <c r="O45">
-        <v>6.7062622530000002</v>
+        <v>4.9056310139999999</v>
       </c>
       <c r="P45">
-        <v>58.59190426</v>
+        <v>36.437753440000002</v>
       </c>
       <c r="Q45">
-        <v>24.337806520000001</v>
+        <v>33.968589559999998</v>
       </c>
       <c r="R45">
-        <v>6.2871595100000004</v>
+        <v>6.5750179839999996</v>
       </c>
       <c r="S45">
-        <v>9.4796660460000002</v>
+        <v>4.3813492370000002</v>
       </c>
       <c r="T45">
-        <v>44.331919970000001</v>
+        <v>24.060362529999999</v>
       </c>
       <c r="U45">
-        <v>14.25998429</v>
+        <v>12.377390910000001</v>
       </c>
       <c r="V45">
-        <v>38.804702710000001</v>
+        <v>59.383017420000002</v>
       </c>
       <c r="W45">
-        <v>2.3566000640000002</v>
+        <v>3.996122518</v>
       </c>
       <c r="X45">
-        <v>0.246792965</v>
+        <v>0.183106624</v>
       </c>
       <c r="Y45">
-        <v>20.118786759999999</v>
+        <v>14.71689304</v>
       </c>
       <c r="Z45">
-        <v>6.4714901449999997</v>
+        <v>7.5708226749999996</v>
       </c>
       <c r="AA45">
-        <v>17.61041569</v>
+        <v>36.322541479999998</v>
       </c>
       <c r="AB45">
-        <v>1.069476219</v>
+        <v>2.4442901730000002</v>
       </c>
       <c r="AC45">
         <v>0.112</v>
       </c>
       <c r="AD45">
-        <v>-0.629023471</v>
+        <v>-1.613734727</v>
       </c>
       <c r="AE45">
-        <v>-0.15897987199999999</v>
+        <v>-0.27725127399999999</v>
       </c>
     </row>
     <row r="46" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A46">
-        <v>44</v>
+        <v>3</v>
       </c>
       <c r="B46" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="C46">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D46" t="s">
         <v>34</v>
@@ -4953,55 +4953,55 @@
         <v>790.1</v>
       </c>
       <c r="O46">
-        <v>6.2861622239999999</v>
+        <v>5</v>
       </c>
       <c r="P46">
-        <v>30.096331939999999</v>
+        <v>70</v>
       </c>
       <c r="Q46">
-        <v>47.51337024</v>
+        <v>10</v>
       </c>
       <c r="R46">
-        <v>8.5863137839999997</v>
+        <v>3.75</v>
       </c>
       <c r="S46">
-        <v>1.5630278559999999</v>
+        <v>41.813333329999999</v>
       </c>
       <c r="T46">
-        <v>15.79655032</v>
+        <v>63</v>
       </c>
       <c r="U46">
-        <v>14.299781619999999</v>
+        <v>7</v>
       </c>
       <c r="V46">
-        <v>63.90151977</v>
+        <v>28.875</v>
       </c>
       <c r="W46">
-        <v>5.9083330370000002</v>
+        <v>0.65459999999999996</v>
       </c>
       <c r="X46">
-        <v>9.3815250000000003E-2</v>
+        <v>0.47039999999999998</v>
       </c>
       <c r="Y46">
-        <v>18.858486670000001</v>
+        <v>15</v>
       </c>
       <c r="Z46">
-        <v>17.07159068</v>
+        <v>1.6666666670000001</v>
       </c>
       <c r="AA46">
-        <v>76.287919500000001</v>
+        <v>6.875</v>
       </c>
       <c r="AB46">
-        <v>7.053579268</v>
+        <v>0.155857143</v>
       </c>
       <c r="AC46">
         <v>0.112</v>
       </c>
       <c r="AD46">
-        <v>-1.5549625840000001</v>
+        <v>-0.47433730600000001</v>
       </c>
       <c r="AE46">
-        <v>-0.24728119900000001</v>
+        <v>-0.373801314</v>
       </c>
     </row>
     <row r="47" spans="1:31" x14ac:dyDescent="0.3">
@@ -5931,8 +5931,8 @@
       <c r="AC100" s="4"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AE26">
-    <sortCondition ref="A2:A26"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AE100">
+    <sortCondition descending="1" ref="AE2:AE100"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>